<commit_message>
Docs: tracker and test report point at PR #309 and migration 0123
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gig-bank-payouts-2026-10/RIDER_BANK_PAYOUTS_TRACKER_2026-10-31.xlsx
+++ b/docs/gig-bank-payouts-2026-10/RIDER_BANK_PAYOUTS_TRACKER_2026-10-31.xlsx
@@ -282,7 +282,7 @@
     <t>CI / local</t>
   </si>
   <si>
-    <t>Running</t>
+    <t>Running in CI (PR #309)</t>
   </si>
   <si>
     <t>Pending</t>
@@ -393,13 +393,13 @@
     <t>Branch</t>
   </si>
   <si>
-    <t>feat/gig-bank-payouts (worktree .claude/worktrees/gig-payouts), not pushed</t>
+    <t>feat/gig-bank-payouts — PR #309 into staging (https://github.com/sanjaymorankar-debug/GoKesari/pull/309)</t>
   </si>
   <si>
     <t>Migration</t>
   </si>
   <si>
-    <t>0121_rider_bank_payouts (additive; rollback scripts/rollback-0121.sql). Number clashes with two unmerged 0121s</t>
+    <t>0123_rider_bank_payouts (additive; rollback scripts/rollback-0123.sql)</t>
   </si>
   <si>
     <t>Flags</t>

</xml_diff>